<commit_message>
tweak map legend selection
</commit_message>
<xml_diff>
--- a/src/data/downloads/parl_1919_main_19190214_data.xlsx
+++ b/src/data/downloads/parl_1919_main_19190214_data.xlsx
@@ -5154,7 +5154,7 @@
     <t>File Generated</t>
   </si>
   <si>
-    <t>2026-05-24T18:03:38.217Z</t>
+    <t>2026-05-24T22:28:17.950Z</t>
   </si>
   <si>
     <t>Data Source</t>
@@ -18873,7 +18873,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -48952,7 +48952,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 

</xml_diff>